<commit_message>
Review six supplied Group A papers and update evidence checkpoint
</commit_message>
<xml_diff>
--- a/groups/group-a/evidence/review_workbook.xlsx
+++ b/groups/group-a/evidence/review_workbook.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R321fabd4d0be4fad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="Rdff1dbcb40e7487c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Included" sheetId="3" r:id="Raa29ffc1a74a4ccd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="4" r:id="R8b8b95a3f04d43c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downloads" sheetId="5" r:id="R0c885fdc738a422f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Searches" sheetId="6" r:id="R04351030901b49cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2a120cadc4a7498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R4f0e38b365c74947"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Included" sheetId="3" r:id="R480f3a01907a4fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="4" r:id="R501db9f2d4934ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downloads" sheetId="5" r:id="R35e7947e0149441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Searches" sheetId="6" r:id="Rb5f4f9d0977e4ae0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Received" sheetId="7" r:id="Rfc86454e31cc4e7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -113,7 +114,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="IncludedTable" displayName="IncludedTable" ref="A1:G17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="IncludedTable" displayName="IncludedTable" ref="A1:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Study"/>
     <x:tableColumn id="2" name="Paper"/>
@@ -128,7 +129,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QualityTable" displayName="QualityTable" ref="A1:N17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QualityTable" displayName="QualityTable" ref="A1:N22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Study"/>
     <x:tableColumn id="2" name="Q1"/>
@@ -150,7 +151,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DownloadsTable" displayName="DownloadsTable" ref="A1:F103" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DownloadsTable" displayName="DownloadsTable" ref="A1:F97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Priority"/>
     <x:tableColumn id="2" name="Record"/>
@@ -174,6 +175,20 @@
     <x:tableColumn id="6" name="Imported"/>
     <x:tableColumn id="7" name="Query"/>
     <x:tableColumn id="8" name="Filters"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ReceivedTable" displayName="ReceivedTable" ref="A1:F7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="Record"/>
+    <x:tableColumn id="2" name="Study"/>
+    <x:tableColumn id="3" name="Filename"/>
+    <x:tableColumn id="4" name="Decision"/>
+    <x:tableColumn id="5" name="QA"/>
+    <x:tableColumn id="6" name="Source SHA256"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -431,7 +446,7 @@
         <x:v>Assessed reports</x:v>
       </x:c>
       <x:c r="B7" s="5" t="n">
-        <x:v>22</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
@@ -439,7 +454,7 @@
         <x:v>Pending retrieval</x:v>
       </x:c>
       <x:c r="B8" s="5" t="n">
-        <x:v>102</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -447,7 +462,7 @@
         <x:v>Accepted studies</x:v>
       </x:c>
       <x:c r="B9" s="5" t="n">
-        <x:v>16</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -455,7 +470,7 @@
         <x:v>Full-text exclusions</x:v>
       </x:c>
       <x:c r="B10" s="5" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -714,19 +729,21 @@
       <x:c r="B7" s="2" t="str">
         <x:v>GA-P0006</x:v>
       </x:c>
-      <x:c r="C7" s="2" t="str"/>
+      <x:c r="C7" s="2" t="str">
+        <x:v>GA-S017</x:v>
+      </x:c>
       <x:c r="D7" s="2" t="str">
         <x:v>VastPipe: A High-Throughput Inference System via Adaptive Space-Division Multiplexing for Diverse Accelerators</x:v>
       </x:c>
       <x:c r="E7" s="2" t="str">
-        <x:v>pending</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="F7" s="2" t="str">
-        <x:v>abstract</x:v>
+        <x:v>full_text</x:v>
       </x:c>
       <x:c r="G7" s="2" t="str"/>
       <x:c r="H7" s="2" t="str">
-        <x:v>Public publisher metadata/abstract examined; full text unavailable. Local inference sharing/assigned mechanism must be checked before acceptance.</x:v>
+        <x:v>Protocol7.2: explicit pairs of inference services share an A100 using MPS, with local throughput comparators. NPU/cluster scope alone would not qualify. Include only local GPU inference evidence, not the main 1000-NPU cluster results. Offline Q-table assumes relatively stable request mix; GPU-specific quotas, repetitions and variance unresolved. Chart bars are not preserved in Markdown. Preliminary ICCD2021 report is linked as an unassessed version lead.</x:v>
       </x:c>
       <x:c r="I7" s="2" t="str">
         <x:v>Springer</x:v>
@@ -735,7 +752,7 @@
         <x:v>SPR-MASTER</x:v>
       </x:c>
       <x:c r="K7" s="2" t="str">
-        <x:v>not_retrieved</x:v>
+        <x:v>retrieved</x:v>
       </x:c>
       <x:c r="L7" s="2" t="str">
         <x:v>https://link.springer.com/article/10.1007/s11390-024-3773-5</x:v>
@@ -990,19 +1007,21 @@
       <x:c r="B15" s="2" t="str">
         <x:v>GA-P0014</x:v>
       </x:c>
-      <x:c r="C15" s="2" t="str"/>
+      <x:c r="C15" s="2" t="str">
+        <x:v>GA-S019</x:v>
+      </x:c>
       <x:c r="D15" s="2" t="str">
         <x:v>Dyna-P: placement-aware dynamic partitioning for lightweight applications with modern GPUs</x:v>
       </x:c>
       <x:c r="E15" s="2" t="str">
-        <x:v>pending</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="F15" s="2" t="str">
-        <x:v>abstract</x:v>
+        <x:v>full_text</x:v>
       </x:c>
       <x:c r="G15" s="2" t="str"/>
       <x:c r="H15" s="2" t="str">
-        <x:v>Public publisher metadata/abstract examined; full text unavailable. Local inference sharing/assigned mechanism must be checked before acceptance.</x:v>
+        <x:v>Protocol7.2: identifiable concurrent inference jobs on MIG partitions; single-A30 local sensitivity/scalability strata in4.2/4.3.1 independently support inclusion. Retain one-GPU inference strata separately from two-GPU aggregate and cluster simulation. JCT/makespan/STP cannot replace request-tail latency or goodput. Reconfiguration can stop/restart active jobs; neither architectural MIG claims nor OOM avoidance prove hostile isolation. Model labels/parameter counts and corrupted overhead fraction require caution.</x:v>
       </x:c>
       <x:c r="I15" s="2" t="str">
         <x:v>Springer</x:v>
@@ -1011,7 +1030,7 @@
         <x:v>SPR-MASTER</x:v>
       </x:c>
       <x:c r="K15" s="2" t="str">
-        <x:v>not_retrieved</x:v>
+        <x:v>retrieved</x:v>
       </x:c>
       <x:c r="L15" s="2" t="str">
         <x:v>https://link.springer.com/article/10.1007/s10586-025-05284-2</x:v>
@@ -1812,19 +1831,21 @@
       <x:c r="B38" s="2" t="str">
         <x:v>GA-P0037</x:v>
       </x:c>
-      <x:c r="C38" s="2" t="str"/>
+      <x:c r="C38" s="2" t="str">
+        <x:v>GA-S018</x:v>
+      </x:c>
       <x:c r="D38" s="2" t="str">
-        <x:v>ArkGPU: enabling applications’ high-goodput co-location execution on multitasking GPUs</x:v>
+        <x:v>ArkGPU: enabling applications' high-goodput co-location execution on multitasking GPUs</x:v>
       </x:c>
       <x:c r="E38" s="2" t="str">
-        <x:v>pending</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="F38" s="2" t="str">
-        <x:v>abstract</x:v>
+        <x:v>full_text</x:v>
       </x:c>
       <x:c r="G38" s="2" t="str"/>
       <x:c r="H38" s="2" t="str">
-        <x:v>Public publisher metadata/abstract examined; full text unavailable. Local inference sharing/assigned mechanism must be checked before acceptance.</x:v>
+        <x:v>Protocol7.2 mixed-workload exception: LC inference-specific outcomes from local inference/training co-location test API control of BE resource interference. Transfer limited to this priority mix. Mixed inference/training qualifies via explicit inference p99/QPS and workload transfer rationale; it does not establish inference-only performance. Polling/API sleeps can add delay; BE checkpoint/restart affects costs. Huge goodput ratios can have near-zero baseline yield. Repetitions/variance and chart coordinates unresolved.</x:v>
       </x:c>
       <x:c r="I38" s="2" t="str">
         <x:v>Springer</x:v>
@@ -1833,7 +1854,7 @@
         <x:v>SPR-MASTER</x:v>
       </x:c>
       <x:c r="K38" s="2" t="str">
-        <x:v>not_retrieved</x:v>
+        <x:v>retrieved</x:v>
       </x:c>
       <x:c r="L38" s="2" t="str">
         <x:v>https://link.springer.com/article/10.1007/s42514-023-00154-y</x:v>
@@ -25161,14 +25182,16 @@
         <x:v>Microsecond-scale Preemption for Concurrent GPU-accelerated DNN Inferences</x:v>
       </x:c>
       <x:c r="E691" s="2" t="str">
-        <x:v>accepted</x:v>
+        <x:v>excluded</x:v>
       </x:c>
       <x:c r="F691" s="2" t="str">
         <x:v>full_text</x:v>
       </x:c>
-      <x:c r="G691" s="2" t="str"/>
+      <x:c r="G691" s="2" t="str">
+        <x:v>E8</x:v>
+      </x:c>
       <x:c r="H691" s="2" t="str">
-        <x:v>Peer-reviewed primary report; local concurrent inference or explicit transferable inference co-location; source-anchored outcomes. Main platform AMD; TOCS extension awaits version assessment.</x:v>
+        <x:v>Less complete OSDI2022 report of GA-S001; journal GA-X007 explicitly extends it with NVIDIA implementation/evaluation. Retained as linked companion, not a second study.</x:v>
       </x:c>
       <x:c r="I691" s="2" t="str">
         <x:v>Supplementary web / venue / author</x:v>
@@ -25766,19 +25789,21 @@
       <x:c r="B708" s="2" t="str">
         <x:v>GA-PX005</x:v>
       </x:c>
-      <x:c r="C708" s="2" t="str"/>
+      <x:c r="C708" s="2" t="str">
+        <x:v>GA-S020</x:v>
+      </x:c>
       <x:c r="D708" s="2" t="str">
         <x:v>iGniter: Interference-Aware GPU Resource Provisioning for Predictable DNN Inference in the Cloud</x:v>
       </x:c>
       <x:c r="E708" s="2" t="str">
-        <x:v>pending</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="F708" s="2" t="str">
-        <x:v>abstract</x:v>
+        <x:v>full_text</x:v>
       </x:c>
       <x:c r="G708" s="2" t="str"/>
       <x:c r="H708" s="2" t="str">
-        <x:v>Verified published TPDS study; publisher unavailable; arXiv PDF retrieval failed.</x:v>
+        <x:v>Protocol7.2: local co-located MPS inference measurements and quota configurations identifiable; fleet allocation/cost is a distinct engineering outcome. Constant arrivals and four vision models limit bursty/LLM transfer. Negligible PCIe contention assumption can underpredict AlexNet; baselines modified. Steady-state/post-correction SLO success is not an unconditional guarantee; shadow standby incurs capacity/memory costs. Chart bars/latency traces unavailable in Markdown.</x:v>
       </x:c>
       <x:c r="I708" s="2" t="str">
         <x:v>Supplementary web / publisher</x:v>
@@ -25787,7 +25812,7 @@
         <x:v>SUP-SELECTED</x:v>
       </x:c>
       <x:c r="K708" s="2" t="str">
-        <x:v>not_retrieved</x:v>
+        <x:v>retrieved</x:v>
       </x:c>
       <x:c r="L708" s="2" t="str">
         <x:v>https://doi.org/10.1109/TPDS.2022.3232715</x:v>
@@ -25800,19 +25825,21 @@
       <x:c r="B709" s="2" t="str">
         <x:v>GA-PX006</x:v>
       </x:c>
-      <x:c r="C709" s="2" t="str"/>
+      <x:c r="C709" s="2" t="str">
+        <x:v>GA-S021</x:v>
+      </x:c>
       <x:c r="D709" s="2" t="str">
-        <x:v>InferFair</x:v>
+        <x:v>InferFair: Towards QoS-aware scheduling for performance isolation guarantee in heterogeneous model serving systems</x:v>
       </x:c>
       <x:c r="E709" s="2" t="str">
-        <x:v>pending</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="F709" s="2" t="str">
-        <x:v>abstract</x:v>
+        <x:v>full_text</x:v>
       </x:c>
       <x:c r="G709" s="2" t="str"/>
       <x:c r="H709" s="2" t="str">
-        <x:v>ScienceDirect 403; full-text eligibility and metadata require verification.</x:v>
+        <x:v>Protocol7.2: local heterogeneous inference scheduling and sharing comparators provide measurable goodput/fairness outcomes, independent of four-GPU replay. Two-column Markdown interleaves algorithms/prose; use labelled Table3 rows and sections, not scrambled formulas. Repetitions/variance and software versions unresolved. MAF trace has minute-level invocation counts; cross-study batching and isolation definitions differ.</x:v>
       </x:c>
       <x:c r="I709" s="2" t="str">
         <x:v>Supplementary web / publisher</x:v>
@@ -25821,7 +25848,7 @@
         <x:v>SUP-SELECTED</x:v>
       </x:c>
       <x:c r="K709" s="2" t="str">
-        <x:v>not_retrieved</x:v>
+        <x:v>retrieved</x:v>
       </x:c>
       <x:c r="L709" s="2" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0167739X23003187</x:v>
@@ -25838,17 +25865,17 @@
         <x:v>GA-S001</x:v>
       </x:c>
       <x:c r="D710" s="2" t="str">
-        <x:v>Real-time Work-conserving GPU Scheduling for DNN Inference</x:v>
+        <x:v>Real-time, Work-conserving GPU Scheduling for Concurrent DNN Inference</x:v>
       </x:c>
       <x:c r="E710" s="2" t="str">
-        <x:v>pending</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="F710" s="2" t="str">
-        <x:v>abstract</x:v>
+        <x:v>full_text</x:v>
       </x:c>
       <x:c r="G710" s="2" t="str"/>
       <x:c r="H710" s="2" t="str">
-        <x:v>Related REEF journal report; assess completeness before replacing conference extraction; never count twice.</x:v>
+        <x:v>Protocol7.2/9: complete peer-reviewed extension explicitly links OSDI2022; new NVIDIA implementation/evaluation and limitations justify preferred version without adding a study. Explicit OSDI2022 extension; select journal as preferred report and retain GA-S001 once. Requires deterministic/stateless kernels; closed-source comparison omits padding. Memory assumed sufficient; bandwidth contention and input-shape profiling limits. Printed publication date differs from some issue-year indexing; recorded2025 follows supplied copy and is in cutoff either way.</x:v>
       </x:c>
       <x:c r="I710" s="2" t="str">
         <x:v>Supplementary web / publisher</x:v>
@@ -25857,7 +25884,7 @@
         <x:v>SUP-SELECTED</x:v>
       </x:c>
       <x:c r="K710" s="2" t="str">
-        <x:v>not_retrieved</x:v>
+        <x:v>retrieved</x:v>
       </x:c>
       <x:c r="L710" s="2" t="str">
         <x:v>https://doi.org/10.1145/3768622</x:v>
@@ -25866,7 +25893,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75f48a502ff142d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5a430e8f2f44b4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25915,19 +25942,19 @@
         <x:v>reef</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
-        <x:v>Temporal preemption</x:v>
+        <x:v>Reset-based temporal preemption + dynamic kernel padding; NVIDIA binary instrumentation</x:v>
       </x:c>
       <x:c r="D2" s="2" t="str">
-        <x:v>https://www.usenix.org/system/files/osdi22-han.pdf</x:v>
+        <x:v>https://doi.org/10.1145/3768622</x:v>
       </x:c>
       <x:c r="E2" s="2" t="str">
-        <x:v>PDF pp11-12; sections7.1-7.2; Fig11</x:v>
+        <x:v>Article pp1:23-1:24,1:31-1:34; sections6.2,6.6,7; Figs28-29; Markdown lines1111-1180,1600-1820</x:v>
       </x:c>
       <x:c r="F2" s="2" t="str">
-        <x:v>DISB-A: RT overhead 0.5% vs RT-only; throughput 1.60x sequential.</x:v>
+        <x:v>GV100 PyTorch DISB-C: Orion p99 normalized latency1.17x vs Reef below1.05x; normalized total throughput0.97x vs1.14x(Fig29). TensorRT comparison trades throughput: mean1.21x Triton vs1.11x Reef(Fig28). All ratios retain model-solo normalization; do not mix engines/AMD strata.</x:v>
       </x:c>
       <x:c r="G2" s="2" t="str">
-        <x:v>Main platform AMD; TOCS extension awaits version assessment.</x:v>
+        <x:v>Explicit OSDI2022 extension; select journal as preferred report and retain GA-S001 once. Requires deterministic/stateless kernels; closed-source comparison omits padding. Memory assumed sufficient; bandwidth contention and input-shape profiling limits. Printed publication date differs from some issue-year indexing; recorded2025 follows supplied copy and is in cutoff either way.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="95" customHeight="1">
@@ -26275,10 +26302,125 @@
         <x:v>Local slice evidence only; multi-server scaling separate; isolation properties described, not attack-tested.</x:v>
       </x:c>
     </x:row>
+    <x:row r="18" ht="95" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>GA-S017</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>vastpipe</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>MPS adaptive quotas; separate AMD CU-mask stratum</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>https://doi.org/10.1007/s11390-024-3773-5</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="str">
+        <x:v>Published pp457-459; sections6.7-6.9; Figs14-16; uploaded Markdown lines1150-1290</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="str">
+        <x:v>A100 VGG16+GoogLeNet: throughput 2.7x no MPS and 1.5x default MPS; not a universal average or p99 result. NLP/CV mean 2.43x no MPS, 1.45x default MPS. MI100 mean 1.89x no mask, 1.24x default mask.</x:v>
+      </x:c>
+      <x:c r="G18" s="2" t="str">
+        <x:v>Include only local GPU inference evidence, not the main 1000-NPU cluster results. Offline Q-table assumes relatively stable request mix; GPU-specific quotas, repetitions and variance unresolved. Chart bars are not preserved in Markdown. Preliminary ICCD2021 report is linked as an unassessed version lead.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="95" customHeight="1">
+      <x:c r="A19" s="2" t="str">
+        <x:v>GA-S018</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>arkgpu</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>CUDA API interception + NVML monitoring and admission throttling</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>https://doi.org/10.1007/s42514-023-00154-y</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="str">
+        <x:v>Published pp313-319; sections4.3,5.1-5.4; Table3; Figs14-21; Markdown lines920-1360</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="str">
+        <x:v>Section5.2 reports all30 tested pairs satisfy the 2x-solo p99 QoS target with ArkGPU. Low-contention pairs can lose about5% QPS from throttling. Four-GPU app-mix goodput gains94.98% vs k8s-native and38.65% vs MPS are separate system-level results.</x:v>
+      </x:c>
+      <x:c r="G19" s="2" t="str">
+        <x:v>Mixed inference/training qualifies via explicit inference p99/QPS and workload transfer rationale; it does not establish inference-only performance. Polling/API sleeps can add delay; BE checkpoint/restart affects costs. Huge goodput ratios can have near-zero baseline yield. Repetitions/variance and chart coordinates unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="95" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>GA-S019</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>dynap</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>MIG dynamic placement/reconfiguration with reconfiguration-last policy</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="str">
+        <x:v>https://doi.org/10.1007/s10586-025-05284-2</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="str">
+        <x:v>PDF pp11-16; sections4.1-4.3.2; Table2; Figs8-13; Markdown lines700-865</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="str">
+        <x:v>Single-A30 batch experiments: smaller partitions increase concurrency but can increase mean JCT; not online p99 evidence. Fig8 broader job set reports39.03% lower makespan vs StaCon,12.14% vs MISO and14.7% higher normalized STP vs StaCon. Prediction-error sensitivity:15% perturbation adds8.09% makespan.</x:v>
+      </x:c>
+      <x:c r="G20" s="2" t="str">
+        <x:v>Retain one-GPU inference strata separately from two-GPU aggregate and cluster simulation. JCT/makespan/STP cannot replace request-tail latency or goodput. Reconfiguration can stop/restart active jobs; neither architectural MIG claims nor OOM avoidance prove hostile isolation. Model labels/parameter counts and corrupted overhead fraction require caution.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="95" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>GA-S020</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>igniter</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>MPS active-thread quotas + interference-aware batch/provisioning and shadow process</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="str">
+        <x:v>https://doi.org/10.1109/TPDS.2022.3232715</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="str">
+        <x:v>Published pp820-824; sections4.2,5.1-5.4; Figs13-18; Markdown lines938-1245</x:v>
+      </x:c>
+      <x:c r="F21" s="2" t="str">
+        <x:v>Local four-model latency prediction error1.53%-5.02%(Fig13). Fig14 deployment: iGniter6 GPUs/0 SLO violations vs gpu-lets+8/3,FFD+5/10,GSLICE+6/3;25% lower hourly instance cost vs gpu-lets+, not25% higher local utilization. Fig17 shows an initial p99 violation before shadow-process recovery.</x:v>
+      </x:c>
+      <x:c r="G21" s="2" t="str">
+        <x:v>Constant arrivals and four vision models limit bursty/LLM transfer. Negligible PCIe contention assumption can underpredict AlexNet; baselines modified. Steady-state/post-correction SLO success is not an unconditional guarantee; shadow standby incurs capacity/memory costs. Chart bars/latency traces unavailable in Markdown.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="95" customHeight="1">
+      <x:c r="A22" s="2" t="str">
+        <x:v>GA-S021</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>inferfair</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>Temporal SLO-aware scheduling + feedback goodput balancing; MPS comparator</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/pii/S0167739X23003187</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="str">
+        <x:v>Published pp17-18; sections5.1-5.4; Table3; Eq2; Markdown lines718-899</x:v>
+      </x:c>
+      <x:c r="F22" s="2" t="str">
+        <x:v>Local Table3 load3:1:2: unfairness1.05 vs Clockwork1.50; SLO goodput524.29 vs457.24req/s. Other load ratios give smaller differences. Local unfairness is max/min model slowdown(Eq2), not p99 or security. Four-GPU MAF outcome kept separate.</x:v>
+      </x:c>
+      <x:c r="G22" s="2" t="str">
+        <x:v>Two-column Markdown interleaves algorithms/prose; use labelled Table3 rows and sections, not scrambled formulas. Repetitions/variance and software versions unresolved. MAF trace has minute-level invocation counts; cross-study batching and isolation definitions differ.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R020d50af52a5434d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11fb79c6e4674bd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26364,7 +26506,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F2" s="2" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="2" t="n">
         <x:v>1</x:v>
@@ -26373,24 +26515,24 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="I2" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="J2" s="2" t="n">
         <x:v>1</x:v>
-      </x:c>
-      <x:c r="J2" s="2" t="n">
-        <x:v>0.5</x:v>
       </x:c>
       <x:c r="K2" s="2" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L2" s="2" t="n">
         <x:f>SUM(B2:K2)</x:f>
-        <x:v>8</x:v>
+        <x:v>8.5</x:v>
       </x:c>
       <x:c r="M2" s="2" t="str">
         <x:f>IF(L2&gt;=8,"high",IF(L2&gt;=6,"moderate","low"))</x:f>
         <x:v>high</x:v>
       </x:c>
       <x:c r="N2" s="2" t="str">
-        <x:v>PDF pp11-12; sections7.1-7.2; Fig11</x:v>
+        <x:v>Article pp1:23-1:24,1:31-1:34; sections6.2,6.6,7; Figs28-29; Markdown lines1111-1180,1600-1820</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -27083,10 +27225,240 @@
         <x:v>HTML Multi-model Scaling/Fig10; Triton implementation; limitations</x:v>
       </x:c>
     </x:row>
+    <x:row r="18" ht="48" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>GA-S017</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G18" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H18" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="J18" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="K18" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="L18" s="2" t="n">
+        <x:f>SUM(B18:K18)</x:f>
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="M18" s="2" t="str">
+        <x:f>IF(L18&gt;=8,"high",IF(L18&gt;=6,"moderate","low"))</x:f>
+        <x:v>moderate</x:v>
+      </x:c>
+      <x:c r="N18" s="2" t="str">
+        <x:v>Published pp457-459; sections6.7-6.9; Figs14-16; uploaded Markdown lines1150-1290</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="48" customHeight="1">
+      <x:c r="A19" s="2" t="str">
+        <x:v>GA-S018</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G19" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H19" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="J19" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="K19" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="L19" s="2" t="n">
+        <x:f>SUM(B19:K19)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="M19" s="2" t="str">
+        <x:f>IF(L19&gt;=8,"high",IF(L19&gt;=6,"moderate","low"))</x:f>
+        <x:v>moderate</x:v>
+      </x:c>
+      <x:c r="N19" s="2" t="str">
+        <x:v>Published pp313-319; sections4.3,5.1-5.4; Table3; Figs14-21; Markdown lines920-1360</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="48" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>GA-S019</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G20" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H20" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="I20" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="J20" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="K20" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="L20" s="2" t="n">
+        <x:f>SUM(B20:K20)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="M20" s="2" t="str">
+        <x:f>IF(L20&gt;=8,"high",IF(L20&gt;=6,"moderate","low"))</x:f>
+        <x:v>moderate</x:v>
+      </x:c>
+      <x:c r="N20" s="2" t="str">
+        <x:v>PDF pp11-16; sections4.1-4.3.2; Table2; Figs8-13; Markdown lines700-865</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="48" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>GA-S020</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F21" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I21" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="J21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K21" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L21" s="2" t="n">
+        <x:f>SUM(B21:K21)</x:f>
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="M21" s="2" t="str">
+        <x:f>IF(L21&gt;=8,"high",IF(L21&gt;=6,"moderate","low"))</x:f>
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="N21" s="2" t="str">
+        <x:v>Published pp820-824; sections4.2,5.1-5.4; Figs13-18; Markdown lines938-1245</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="48" customHeight="1">
+      <x:c r="A22" s="2" t="str">
+        <x:v>GA-S021</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F22" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G22" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H22" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="I22" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J22" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="K22" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="L22" s="2" t="n">
+        <x:f>SUM(B22:K22)</x:f>
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="M22" s="2" t="str">
+        <x:f>IF(L22&gt;=8,"high",IF(L22&gt;=6,"moderate","low"))</x:f>
+        <x:v>moderate</x:v>
+      </x:c>
+      <x:c r="N22" s="2" t="str">
+        <x:v>Published pp17-18; sections5.1-5.4; Table3; Eq2; Markdown lines718-899</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d8bafa980f54821"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cde3691092e4ecf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27125,19 +27497,19 @@
     </x:row>
     <x:row r="2" ht="65" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>unavailable_not_requested_again</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>GA-X005</x:v>
+        <x:v>GA-R0011</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
-        <x:v>iGniter: Interference-Aware GPU Resource Provisioning for Predictable DNN Inference in the Cloud</x:v>
+        <x:v>GhostWriter: Exploiting GPU-Cache Contention to Steal and Steer Multi-tenant Large-Language-Model Inference</x:v>
       </x:c>
       <x:c r="D2" s="2" t="str">
-        <x:v>IEEE Xplore</x:v>
+        <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E2" s="2" t="str">
-        <x:v>https://doi.org/10.1109/TPDS.2022.3232715</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-032-16342-4_8</x:v>
       </x:c>
       <x:c r="F2" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27145,19 +27517,19 @@
     </x:row>
     <x:row r="3" ht="65" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>unavailable_not_requested_again</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
-        <x:v>GA-R0011</x:v>
+        <x:v>GA-R0004</x:v>
       </x:c>
       <x:c r="C3" s="2" t="str">
-        <x:v>GhostWriter: Exploiting GPU-Cache Contention to Steal and Steer Multi-tenant Large-Language-Model Inference</x:v>
+        <x:v>HAS-GPU: Efficient Hybrid Auto-scaling with Fine-Grained GPU Allocation for SLO-Aware Serverless Inferences</x:v>
       </x:c>
       <x:c r="D3" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E3" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-032-16342-4_8</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-99854-6_11</x:v>
       </x:c>
       <x:c r="F3" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27165,19 +27537,19 @@
     </x:row>
     <x:row r="4" ht="65" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>unavailable_not_requested_again</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
-        <x:v>GA-R0004</x:v>
+        <x:v>GA-R0292</x:v>
       </x:c>
       <x:c r="C4" s="2" t="str">
-        <x:v>HAS-GPU: Efficient Hybrid Auto-scaling with Fine-Grained GPU Allocation for SLO-Aware Serverless Inferences</x:v>
+        <x:v>A Close Look at Multi-tenant Parallel CNN Inference for Autonomous Driving</x:v>
       </x:c>
       <x:c r="D4" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E4" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-99854-6_11</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-79478-1_8</x:v>
       </x:c>
       <x:c r="F4" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27185,19 +27557,19 @@
     </x:row>
     <x:row r="5" ht="65" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>unavailable_not_requested_again</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>GA-R0292</x:v>
+        <x:v>GA-R0009</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>A Close Look at Multi-tenant Parallel CNN Inference for Autonomous Driving</x:v>
+        <x:v>vGPU Performance Testing Framework for Large Model Inference</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E5" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-79478-1_8</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-981-96-8728-2_35</x:v>
       </x:c>
       <x:c r="F5" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27205,19 +27577,19 @@
     </x:row>
     <x:row r="6" ht="65" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B6" s="2" t="str">
-        <x:v>GA-R0006</x:v>
+        <x:v>GA-R0001</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
-        <x:v>VastPipe: A High-Throughput Inference System via Adaptive Space-Division Multiplexing for Diverse Accelerators</x:v>
+        <x:v>A comprehensive evaluation of spatial co-execution on GPUs using MPS and MIG technologies</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E6" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11390-024-3773-5</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11227-026-08312-z</x:v>
       </x:c>
       <x:c r="F6" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27225,19 +27597,19 @@
     </x:row>
     <x:row r="7" ht="65" customHeight="1">
       <x:c r="A7" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B7" s="2" t="str">
-        <x:v>GA-R0014</x:v>
+        <x:v>GA-R0002</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
-        <x:v>Dyna-P: placement-aware dynamic partitioning for lightweight applications with modern GPUs</x:v>
+        <x:v>Oltunes: Online learning-based auto-tuning system for DL inference in heterogeneous GPU cluster</x:v>
       </x:c>
       <x:c r="D7" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E7" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10586-025-05284-2</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s10586-025-05216-0</x:v>
       </x:c>
       <x:c r="F7" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27245,19 +27617,19 @@
     </x:row>
     <x:row r="8" ht="65" customHeight="1">
       <x:c r="A8" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
-        <x:v>GA-X006</x:v>
+        <x:v>GA-R0003</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
-        <x:v>InferFair</x:v>
+        <x:v>MuxFlow: efficient GPU sharing in production-level clusters with more than 10000 GPUs</x:v>
       </x:c>
       <x:c r="D8" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E8" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/pii/S0167739X23003187</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11432-024-4227-2</x:v>
       </x:c>
       <x:c r="F8" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27265,19 +27637,19 @@
     </x:row>
     <x:row r="9" ht="65" customHeight="1">
       <x:c r="A9" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
-        <x:v>GA-X007</x:v>
+        <x:v>GA-R0005</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>Real-time Work-conserving GPU Scheduling for DNN Inference</x:v>
+        <x:v>Understanding GPU-Level Bottlenecks in Large Language Model Inference</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
-        <x:v>ACM DL</x:v>
+        <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E9" s="2" t="str">
-        <x:v>https://doi.org/10.1145/3768622</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-032-27448-9_18</x:v>
       </x:c>
       <x:c r="F9" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27285,19 +27657,19 @@
     </x:row>
     <x:row r="10" ht="65" customHeight="1">
       <x:c r="A10" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>GA-R0009</x:v>
+        <x:v>GA-R0007</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
-        <x:v>vGPU Performance Testing Framework for Large Model Inference</x:v>
+        <x:v>Design and Operation of Elastic GPU-Pooling on Campus</x:v>
       </x:c>
       <x:c r="D10" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E10" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-981-96-8728-2_35</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-99854-6_27</x:v>
       </x:c>
       <x:c r="F10" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27305,19 +27677,19 @@
     </x:row>
     <x:row r="11" ht="65" customHeight="1">
       <x:c r="A11" s="2" t="str">
-        <x:v>requested_max10</x:v>
+        <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B11" s="2" t="str">
-        <x:v>GA-R0037</x:v>
+        <x:v>GA-R0008</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
-        <x:v>ArkGPU: enabling applications’ high-goodput co-location execution on multitasking GPUs</x:v>
+        <x:v>SpecInF: Exploiting Idle GPU Resources in Distributed DL Training via Speculative Inference Filling</x:v>
       </x:c>
       <x:c r="D11" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E11" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42514-023-00154-y</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-981-96-2830-8_12</x:v>
       </x:c>
       <x:c r="F11" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27328,16 +27700,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B12" s="2" t="str">
-        <x:v>GA-R0001</x:v>
+        <x:v>GA-R0013</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
-        <x:v>A comprehensive evaluation of spatial co-execution on GPUs using MPS and MIG technologies</x:v>
+        <x:v>DRAFAS: Dynamic Resource Allocation for AI-Native Services</x:v>
       </x:c>
       <x:c r="D12" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E12" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11227-026-08312-z</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s10922-025-09962-9</x:v>
       </x:c>
       <x:c r="F12" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27348,16 +27720,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B13" s="2" t="str">
-        <x:v>GA-R0002</x:v>
+        <x:v>GA-R0016</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
-        <x:v>Oltunes: Online learning-based auto-tuning system for DL inference in heterogeneous GPU cluster</x:v>
+        <x:v>Learning to schedule: interference-aware optimization for edge AI inference on shared GPUs</x:v>
       </x:c>
       <x:c r="D13" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E13" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10586-025-05216-0</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11432-025-5051-3</x:v>
       </x:c>
       <x:c r="F13" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27368,16 +27740,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B14" s="2" t="str">
-        <x:v>GA-R0003</x:v>
+        <x:v>GA-R0030</x:v>
       </x:c>
       <x:c r="C14" s="2" t="str">
-        <x:v>MuxFlow: efficient GPU sharing in production-level clusters with more than 10000 GPUs</x:v>
+        <x:v>CoFB: latency-constrained co-scheduling of flows and batches for deep learning inference service on the CPU–GPU system</x:v>
       </x:c>
       <x:c r="D14" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E14" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11432-024-4227-2</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11227-023-05183-6</x:v>
       </x:c>
       <x:c r="F14" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27388,16 +27760,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B15" s="2" t="str">
-        <x:v>GA-R0005</x:v>
+        <x:v>GA-R0038</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
-        <x:v>Understanding GPU-Level Bottlenecks in Large Language Model Inference</x:v>
+        <x:v>Towards Using Partitioned GPU Virtual Functions for Mixture of Experts</x:v>
       </x:c>
       <x:c r="D15" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E15" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-032-27448-9_18</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-90200-0_14</x:v>
       </x:c>
       <x:c r="F15" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27408,16 +27780,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>GA-R0007</x:v>
+        <x:v>GA-R0039</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
-        <x:v>Design and Operation of Elastic GPU-Pooling on Campus</x:v>
+        <x:v>Policy-aware GPU resource allocation for national supercomputing</x:v>
       </x:c>
       <x:c r="D16" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E16" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-99854-6_27</x:v>
+        <x:v>https://link.springer.com/article/10.1038/s41598-026-42625-6</x:v>
       </x:c>
       <x:c r="F16" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27428,16 +27800,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>GA-R0008</x:v>
+        <x:v>GA-R0048</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
-        <x:v>SpecInF: Exploiting Idle GPU Resources in Distributed DL Training via Speculative Inference Filling</x:v>
+        <x:v>MPL-schedule: a dynamic priority-based scheduling scheme for spiking neural networks</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E17" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-981-96-2830-8_12</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11432-025-5044-3</x:v>
       </x:c>
       <x:c r="F17" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27448,16 +27820,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>GA-R0013</x:v>
+        <x:v>GA-R0049</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
-        <x:v>DRAFAS: Dynamic Resource Allocation for AI-Native Services</x:v>
+        <x:v>gCFS: completely fair scheduling on multiple GPUs for improved multi-DNN execution in terms of performance isolation</x:v>
       </x:c>
       <x:c r="D18" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E18" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10922-025-09962-9</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11227-022-04901-w</x:v>
       </x:c>
       <x:c r="F18" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27468,16 +27840,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B19" s="2" t="str">
-        <x:v>GA-R0016</x:v>
+        <x:v>GA-R0067</x:v>
       </x:c>
       <x:c r="C19" s="2" t="str">
-        <x:v>Learning to schedule: interference-aware optimization for edge AI inference on shared GPUs</x:v>
+        <x:v>SLO-Aware DL Job Scheduling for Efficient FPGA-GPU Edge Cloud Computing</x:v>
       </x:c>
       <x:c r="D19" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E19" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11432-025-5051-3</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-50385-6_2</x:v>
       </x:c>
       <x:c r="F19" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27488,16 +27860,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B20" s="2" t="str">
-        <x:v>GA-R0030</x:v>
+        <x:v>GA-R0069</x:v>
       </x:c>
       <x:c r="C20" s="2" t="str">
-        <x:v>CoFB: latency-constrained co-scheduling of flows and batches for deep learning inference service on the CPU–GPU system</x:v>
+        <x:v>KubeGPU: efficient sharing and isolation mechanisms for GPU resource management in container cloud</x:v>
       </x:c>
       <x:c r="D20" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E20" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11227-023-05183-6</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11227-022-04682-2</x:v>
       </x:c>
       <x:c r="F20" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27508,16 +27880,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B21" s="2" t="str">
-        <x:v>GA-R0038</x:v>
+        <x:v>GA-R0070</x:v>
       </x:c>
       <x:c r="C21" s="2" t="str">
-        <x:v>Towards Using Partitioned GPU Virtual Functions for Mixture of Experts</x:v>
+        <x:v>InferONNX: Practical and Privacy-Preserving Machine Learning Inference Using Trusted Execution Environments</x:v>
       </x:c>
       <x:c r="D21" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E21" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-90200-0_14</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-97623-0_2</x:v>
       </x:c>
       <x:c r="F21" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27528,16 +27900,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B22" s="2" t="str">
-        <x:v>GA-R0039</x:v>
+        <x:v>GA-R0081</x:v>
       </x:c>
       <x:c r="C22" s="2" t="str">
-        <x:v>Policy-aware GPU resource allocation for national supercomputing</x:v>
+        <x:v>Smash: A Compression Benchmark with AI Datasets from Remote GPU Virtualization Systems</x:v>
       </x:c>
       <x:c r="D22" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E22" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1038/s41598-026-42625-6</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-15471-3_21</x:v>
       </x:c>
       <x:c r="F22" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27548,16 +27920,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B23" s="2" t="str">
-        <x:v>GA-R0048</x:v>
+        <x:v>GA-R0087</x:v>
       </x:c>
       <x:c r="C23" s="2" t="str">
-        <x:v>MPL-schedule: a dynamic priority-based scheduling scheme for spiking neural networks</x:v>
+        <x:v>Modeling throughput and power consumption for real-time concurrent vision application deployments on edge</x:v>
       </x:c>
       <x:c r="D23" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E23" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11432-025-5044-3</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11554-026-01915-y</x:v>
       </x:c>
       <x:c r="F23" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27568,16 +27940,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B24" s="2" t="str">
-        <x:v>GA-R0049</x:v>
+        <x:v>GA-R0089</x:v>
       </x:c>
       <x:c r="C24" s="2" t="str">
-        <x:v>gCFS: completely fair scheduling on multiple GPUs for improved multi-DNN execution in terms of performance isolation</x:v>
+        <x:v>DELCAS: Deep Reinforcement Learning Based GPU CaaS Packet Scheduling for Stabilizing QoE in 5G Multi-Access Edge Computing</x:v>
       </x:c>
       <x:c r="D24" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E24" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11227-022-04901-w</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-50385-6_5</x:v>
       </x:c>
       <x:c r="F24" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27588,16 +27960,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B25" s="2" t="str">
-        <x:v>GA-R0067</x:v>
+        <x:v>GA-R0092</x:v>
       </x:c>
       <x:c r="C25" s="2" t="str">
-        <x:v>SLO-Aware DL Job Scheduling for Efficient FPGA-GPU Edge Cloud Computing</x:v>
+        <x:v>PYRA: Parallel Yielding Re-activation for Training-Inference Efficient Task Adaptation</x:v>
       </x:c>
       <x:c r="D25" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E25" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-50385-6_2</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-72673-6_25</x:v>
       </x:c>
       <x:c r="F25" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27608,16 +27980,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B26" s="2" t="str">
-        <x:v>GA-R0069</x:v>
+        <x:v>GA-R0117</x:v>
       </x:c>
       <x:c r="C26" s="2" t="str">
-        <x:v>KubeGPU: efficient sharing and isolation mechanisms for GPU resource management in container cloud</x:v>
+        <x:v>Exploring cloud instance options for optimal performance-cost efficiency</x:v>
       </x:c>
       <x:c r="D26" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E26" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11227-022-04682-2</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s10586-025-05702-5</x:v>
       </x:c>
       <x:c r="F26" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27628,16 +28000,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B27" s="2" t="str">
-        <x:v>GA-R0070</x:v>
+        <x:v>GA-R0139</x:v>
       </x:c>
       <x:c r="C27" s="2" t="str">
-        <x:v>InferONNX: Practical and Privacy-Preserving Machine Learning Inference Using Trusted Execution Environments</x:v>
+        <x:v>Dynamic Resource Management for Machine Learning Pipeline Workloads</x:v>
       </x:c>
       <x:c r="D27" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E27" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-97623-0_2</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s42979-023-02101-8</x:v>
       </x:c>
       <x:c r="F27" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27648,16 +28020,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B28" s="2" t="str">
-        <x:v>GA-R0081</x:v>
+        <x:v>GA-R0150</x:v>
       </x:c>
       <x:c r="C28" s="2" t="str">
-        <x:v>Smash: A Compression Benchmark with AI Datasets from Remote GPU Virtualization Systems</x:v>
+        <x:v>Design and implementation of fully distributed heterogeneous resource management system</x:v>
       </x:c>
       <x:c r="D28" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E28" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-15471-3_21</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s10586-025-05154-x</x:v>
       </x:c>
       <x:c r="F28" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27668,16 +28040,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B29" s="2" t="str">
-        <x:v>GA-R0087</x:v>
+        <x:v>GA-R0242</x:v>
       </x:c>
       <x:c r="C29" s="2" t="str">
-        <x:v>Modeling throughput and power consumption for real-time concurrent vision application deployments on edge</x:v>
+        <x:v>Interference-aware execution framework with Co-scheML on GPU clusters</x:v>
       </x:c>
       <x:c r="D29" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E29" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11554-026-01915-y</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s10586-021-03299-z</x:v>
       </x:c>
       <x:c r="F29" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27688,16 +28060,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B30" s="2" t="str">
-        <x:v>GA-R0089</x:v>
+        <x:v>GA-R0249</x:v>
       </x:c>
       <x:c r="C30" s="2" t="str">
-        <x:v>DELCAS: Deep Reinforcement Learning Based GPU CaaS Packet Scheduling for Stabilizing QoE in 5G Multi-Access Edge Computing</x:v>
+        <x:v>AIMSM - A Mechanism to Optimize Systems with Multiple AI Models: A Case Study in Computer Vision for Autonomous Mobile Robots</x:v>
       </x:c>
       <x:c r="D30" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E30" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-50385-6_5</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-73503-5_5</x:v>
       </x:c>
       <x:c r="F30" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27708,16 +28080,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B31" s="2" t="str">
-        <x:v>GA-R0092</x:v>
+        <x:v>GA-R0255</x:v>
       </x:c>
       <x:c r="C31" s="2" t="str">
-        <x:v>PYRA: Parallel Yielding Re-activation for Training-Inference Efficient Task Adaptation</x:v>
+        <x:v>Orchestrated Co-scheduling, Resource Partitioning, and Power Capping on CPU-GPU Heterogeneous Systems via Machine Learning</x:v>
       </x:c>
       <x:c r="D31" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E31" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-72673-6_25</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-21867-5_4</x:v>
       </x:c>
       <x:c r="F31" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27728,16 +28100,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B32" s="2" t="str">
-        <x:v>GA-R0117</x:v>
+        <x:v>GA-R0277</x:v>
       </x:c>
       <x:c r="C32" s="2" t="str">
-        <x:v>Exploring cloud instance options for optimal performance-cost efficiency</x:v>
+        <x:v>Job placement using reinforcement learning in GPU virtualization environment</x:v>
       </x:c>
       <x:c r="D32" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E32" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10586-025-05702-5</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s10586-019-03044-7</x:v>
       </x:c>
       <x:c r="F32" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27748,16 +28120,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B33" s="2" t="str">
-        <x:v>GA-R0139</x:v>
+        <x:v>GA-R0328</x:v>
       </x:c>
       <x:c r="C33" s="2" t="str">
-        <x:v>Dynamic Resource Management for Machine Learning Pipeline Workloads</x:v>
+        <x:v>Euge: Effective Utilization of GPU Resources for Serving DNN-Based Video Analysis</x:v>
       </x:c>
       <x:c r="D33" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E33" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42979-023-02101-8</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-60290-1_40</x:v>
       </x:c>
       <x:c r="F33" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27768,16 +28140,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B34" s="2" t="str">
-        <x:v>GA-R0150</x:v>
+        <x:v>GA-R0370</x:v>
       </x:c>
       <x:c r="C34" s="2" t="str">
-        <x:v>Design and implementation of fully distributed heterogeneous resource management system</x:v>
+        <x:v>Collaborative GPU Preemption via Spatial Multitasking for Efficient GPU Sharing</x:v>
       </x:c>
       <x:c r="D34" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E34" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10586-025-05154-x</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-85665-6_6</x:v>
       </x:c>
       <x:c r="F34" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27788,16 +28160,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B35" s="2" t="str">
-        <x:v>GA-R0242</x:v>
+        <x:v>GA-R0424</x:v>
       </x:c>
       <x:c r="C35" s="2" t="str">
-        <x:v>Interference-aware execution framework with Co-scheML on GPU clusters</x:v>
+        <x:v>On Reverse Engineering Neural Network Implementation on GPU</x:v>
       </x:c>
       <x:c r="D35" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E35" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10586-021-03299-z</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-81645-2_7</x:v>
       </x:c>
       <x:c r="F35" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27808,16 +28180,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B36" s="2" t="str">
-        <x:v>GA-R0249</x:v>
+        <x:v>GA-R0446</x:v>
       </x:c>
       <x:c r="C36" s="2" t="str">
-        <x:v>AIMSM - A Mechanism to Optimize Systems with Multiple AI Models: A Case Study in Computer Vision for Autonomous Mobile Robots</x:v>
+        <x:v>qCUDA-ARM: Virtualization for Embedded GPU Architectures</x:v>
       </x:c>
       <x:c r="D36" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E36" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-73503-5_5</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-38651-1_23</x:v>
       </x:c>
       <x:c r="F36" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27828,16 +28200,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B37" s="2" t="str">
-        <x:v>GA-R0255</x:v>
+        <x:v>GA-R0471</x:v>
       </x:c>
       <x:c r="C37" s="2" t="str">
-        <x:v>Orchestrated Co-scheduling, Resource Partitioning, and Power Capping on CPU-GPU Heterogeneous Systems via Machine Learning</x:v>
+        <x:v>FLARE: Flexibly Sharing Commodity GPUs to Enforce QoS and Improve Utilization</x:v>
       </x:c>
       <x:c r="D37" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E37" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-21867-5_4</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-72789-5_3</x:v>
       </x:c>
       <x:c r="F37" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27848,16 +28220,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B38" s="2" t="str">
-        <x:v>GA-R0277</x:v>
+        <x:v>GA-R0479</x:v>
       </x:c>
       <x:c r="C38" s="2" t="str">
-        <x:v>Job placement using reinforcement learning in GPU virtualization environment</x:v>
+        <x:v>K-Scheduler: dynamic intra-SM multitasking management with execution profiles on GPUs</x:v>
       </x:c>
       <x:c r="D38" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E38" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10586-019-03044-7</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s10586-021-03429-7</x:v>
       </x:c>
       <x:c r="F38" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27868,16 +28240,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B39" s="2" t="str">
-        <x:v>GA-R0328</x:v>
+        <x:v>GA-R0533</x:v>
       </x:c>
       <x:c r="C39" s="2" t="str">
-        <x:v>Euge: Effective Utilization of GPU Resources for Serving DNN-Based Video Analysis</x:v>
+        <x:v>Horus: An Interference-Aware Resource Manager for Deep Learning Systems</x:v>
       </x:c>
       <x:c r="D39" s="2" t="str">
         <x:v>Springer Nature Link</x:v>
       </x:c>
       <x:c r="E39" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-60290-1_40</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-60239-0_33</x:v>
       </x:c>
       <x:c r="F39" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27888,16 +28260,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B40" s="2" t="str">
-        <x:v>GA-R0370</x:v>
+        <x:v>GA-R0591</x:v>
       </x:c>
       <x:c r="C40" s="2" t="str">
-        <x:v>Collaborative GPU Preemption via Spatial Multitasking for Efficient GPU Sharing</x:v>
+        <x:v>GPU Partitioning Mechanisms for Safety-related Applications</x:v>
       </x:c>
       <x:c r="D40" s="2" t="str">
-        <x:v>Springer Nature Link</x:v>
+        <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E40" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-85665-6_6</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11727489/</x:v>
       </x:c>
       <x:c r="F40" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27908,16 +28280,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B41" s="2" t="str">
-        <x:v>GA-R0424</x:v>
+        <x:v>GA-R0592</x:v>
       </x:c>
       <x:c r="C41" s="2" t="str">
-        <x:v>On Reverse Engineering Neural Network Implementation on GPU</x:v>
+        <x:v>Joint Optimization of Resource Allocation and Request Batching for Multi-Tenant Inference Serving on GPU</x:v>
       </x:c>
       <x:c r="D41" s="2" t="str">
-        <x:v>Springer Nature Link</x:v>
+        <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E41" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-81645-2_7</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11223102/</x:v>
       </x:c>
       <x:c r="F41" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27928,16 +28300,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B42" s="2" t="str">
-        <x:v>GA-R0446</x:v>
+        <x:v>GA-R0593</x:v>
       </x:c>
       <x:c r="C42" s="2" t="str">
-        <x:v>qCUDA-ARM: Virtualization for Embedded GPU Architectures</x:v>
+        <x:v>InSS: An Intelligent Scheduling Orchestrator for Multi-GPU Inference With Spatio-Temporal Sharing</x:v>
       </x:c>
       <x:c r="D42" s="2" t="str">
-        <x:v>Springer Nature Link</x:v>
+        <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E42" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-38651-1_23</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10601534/</x:v>
       </x:c>
       <x:c r="F42" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27948,16 +28320,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B43" s="2" t="str">
-        <x:v>GA-R0471</x:v>
+        <x:v>GA-R0595</x:v>
       </x:c>
       <x:c r="C43" s="2" t="str">
-        <x:v>FLARE: Flexibly Sharing Commodity GPUs to Enforce QoS and Improve Utilization</x:v>
+        <x:v>Interference-Aware Latency Prediction With Kernels For Deep Neural Network</x:v>
       </x:c>
       <x:c r="D43" s="2" t="str">
-        <x:v>Springer Nature Link</x:v>
+        <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E43" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-72789-5_3</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10062171/</x:v>
       </x:c>
       <x:c r="F43" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27968,16 +28340,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B44" s="2" t="str">
-        <x:v>GA-R0479</x:v>
+        <x:v>GA-R0596</x:v>
       </x:c>
       <x:c r="C44" s="2" t="str">
-        <x:v>K-Scheduler: dynamic intra-SM multitasking management with execution profiles on GPUs</x:v>
+        <x:v>GPU Overdrive Fault Attacks on Neural Networks</x:v>
       </x:c>
       <x:c r="D44" s="2" t="str">
-        <x:v>Springer Nature Link</x:v>
+        <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E44" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10586-021-03429-7</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9643486/</x:v>
       </x:c>
       <x:c r="F44" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -27988,16 +28360,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B45" s="2" t="str">
-        <x:v>GA-R0533</x:v>
+        <x:v>GA-R0597</x:v>
       </x:c>
       <x:c r="C45" s="2" t="str">
-        <x:v>Horus: An Interference-Aware Resource Manager for Deep Learning Systems</x:v>
+        <x:v>Priority-Aware GPU Co-Scheduling for High Performance Computing</x:v>
       </x:c>
       <x:c r="D45" s="2" t="str">
-        <x:v>Springer Nature Link</x:v>
+        <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E45" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-030-60239-0_33</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11619013/</x:v>
       </x:c>
       <x:c r="F45" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28008,16 +28380,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B46" s="2" t="str">
-        <x:v>GA-R0591</x:v>
+        <x:v>GA-R0598</x:v>
       </x:c>
       <x:c r="C46" s="2" t="str">
-        <x:v>GPU Partitioning Mechanisms for Safety-related Applications</x:v>
+        <x:v>WAGES: Workload-Aware GPU Sharing System for Energy-Efficient Serverless LLM Serving</x:v>
       </x:c>
       <x:c r="D46" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E46" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11727489/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11357986/</x:v>
       </x:c>
       <x:c r="F46" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28028,16 +28400,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B47" s="2" t="str">
-        <x:v>GA-R0592</x:v>
+        <x:v>GA-R0599</x:v>
       </x:c>
       <x:c r="C47" s="2" t="str">
-        <x:v>Joint Optimization of Resource Allocation and Request Batching for Multi-Tenant Inference Serving on GPU</x:v>
+        <x:v>Utilizing Machine Learning Techniques for Worst-Case Execution Time Estimation on GPU Architectures</x:v>
       </x:c>
       <x:c r="D47" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E47" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11223102/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10474357/</x:v>
       </x:c>
       <x:c r="F47" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28048,16 +28420,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B48" s="2" t="str">
-        <x:v>GA-R0593</x:v>
+        <x:v>GA-R0600</x:v>
       </x:c>
       <x:c r="C48" s="2" t="str">
-        <x:v>InSS: An Intelligent Scheduling Orchestrator for Multi-GPU Inference With Spatio-Temporal Sharing</x:v>
+        <x:v>HeShare: Energy-Aware and Efficient Multi-Task GPU Sharing in Heterogeneous GPU-Based Computing Systems</x:v>
       </x:c>
       <x:c r="D48" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E48" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10601534/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11230091/</x:v>
       </x:c>
       <x:c r="F48" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28068,16 +28440,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B49" s="2" t="str">
-        <x:v>GA-R0595</x:v>
+        <x:v>GA-R0601</x:v>
       </x:c>
       <x:c r="C49" s="2" t="str">
-        <x:v>Interference-Aware Latency Prediction With Kernels For Deep Neural Network</x:v>
+        <x:v>Exploring the Diversity of Multiple Job Deployments over GPUs for Efficient Resource Sharing</x:v>
       </x:c>
       <x:c r="D49" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E49" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10062171/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10572198/</x:v>
       </x:c>
       <x:c r="F49" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28088,16 +28460,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B50" s="2" t="str">
-        <x:v>GA-R0596</x:v>
+        <x:v>GA-R0602</x:v>
       </x:c>
       <x:c r="C50" s="2" t="str">
-        <x:v>GPU Overdrive Fault Attacks on Neural Networks</x:v>
+        <x:v>ECML: Improving Efficiency of Machine Learning in Edge Clouds</x:v>
       </x:c>
       <x:c r="D50" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E50" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9643486/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9335804/</x:v>
       </x:c>
       <x:c r="F50" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28108,16 +28480,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B51" s="2" t="str">
-        <x:v>GA-R0597</x:v>
+        <x:v>GA-R0603</x:v>
       </x:c>
       <x:c r="C51" s="2" t="str">
-        <x:v>Priority-Aware GPU Co-Scheduling for High Performance Computing</x:v>
+        <x:v>DistMind: Efficient Resource Disaggregation for Deep Learning Workloads</x:v>
       </x:c>
       <x:c r="D51" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E51" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11619013/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10414009/</x:v>
       </x:c>
       <x:c r="F51" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28128,16 +28500,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B52" s="2" t="str">
-        <x:v>GA-R0598</x:v>
+        <x:v>GA-R0604</x:v>
       </x:c>
       <x:c r="C52" s="2" t="str">
-        <x:v>WAGES: Workload-Aware GPU Sharing System for Energy-Efficient Serverless LLM Serving</x:v>
+        <x:v>Granularity- and Interference-Aware GPU Sharing with MPS</x:v>
       </x:c>
       <x:c r="D52" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E52" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11357986/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10820577/</x:v>
       </x:c>
       <x:c r="F52" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28148,16 +28520,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B53" s="2" t="str">
-        <x:v>GA-R0599</x:v>
+        <x:v>GA-R0605</x:v>
       </x:c>
       <x:c r="C53" s="2" t="str">
-        <x:v>Utilizing Machine Learning Techniques for Worst-Case Execution Time Estimation on GPU Architectures</x:v>
+        <x:v>Machine Learning at the Edge: Efficient Utilization of Limited CPU/GPU Resources by Multiplexing</x:v>
       </x:c>
       <x:c r="D53" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E53" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10474357/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9259361/</x:v>
       </x:c>
       <x:c r="F53" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28168,16 +28540,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B54" s="2" t="str">
-        <x:v>GA-R0600</x:v>
+        <x:v>GA-R0607</x:v>
       </x:c>
       <x:c r="C54" s="2" t="str">
-        <x:v>HeShare: Energy-Aware and Efficient Multi-Task GPU Sharing in Heterogeneous GPU-Based Computing Systems</x:v>
+        <x:v>Towards Deterministic End-to-end Latency for Medical AI Systems in NVIDIA Holoscan</x:v>
       </x:c>
       <x:c r="D54" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E54" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11230091/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10571631/</x:v>
       </x:c>
       <x:c r="F54" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28188,16 +28560,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B55" s="2" t="str">
-        <x:v>GA-R0601</x:v>
+        <x:v>GA-R0608</x:v>
       </x:c>
       <x:c r="C55" s="2" t="str">
-        <x:v>Exploring the Diversity of Multiple Job Deployments over GPUs for Efficient Resource Sharing</x:v>
+        <x:v>DARIS: An Oversubscribed Spatio-Temporal Scheduler for Real-Time DNN Inference on GPUs</x:v>
       </x:c>
       <x:c r="D55" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E55" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10572198/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11132423/</x:v>
       </x:c>
       <x:c r="F55" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28208,16 +28580,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B56" s="2" t="str">
-        <x:v>GA-R0602</x:v>
+        <x:v>GA-R0613</x:v>
       </x:c>
       <x:c r="C56" s="2" t="str">
-        <x:v>ECML: Improving Efficiency of Machine Learning in Edge Clouds</x:v>
+        <x:v>Performance Characterization of LLM Inference under Limited GPU Resources</x:v>
       </x:c>
       <x:c r="D56" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E56" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9335804/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11645315/</x:v>
       </x:c>
       <x:c r="F56" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28228,16 +28600,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B57" s="2" t="str">
-        <x:v>GA-R0603</x:v>
+        <x:v>GA-R0614</x:v>
       </x:c>
       <x:c r="C57" s="2" t="str">
-        <x:v>DistMind: Efficient Resource Disaggregation for Deep Learning Workloads</x:v>
+        <x:v>Characterizing GPU Capacity and Computational Cost in Production AI Inference Using a Replica-Centric Measurement Framework</x:v>
       </x:c>
       <x:c r="D57" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E57" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10414009/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11653193/</x:v>
       </x:c>
       <x:c r="F57" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28248,16 +28620,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B58" s="2" t="str">
-        <x:v>GA-R0604</x:v>
+        <x:v>GA-R0617</x:v>
       </x:c>
       <x:c r="C58" s="2" t="str">
-        <x:v>Granularity- and Interference-Aware GPU Sharing with MPS</x:v>
+        <x:v>Characterizing Multi-Instance GPU for Machine Learning Workloads</x:v>
       </x:c>
       <x:c r="D58" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E58" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10820577/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9835424/</x:v>
       </x:c>
       <x:c r="F58" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28268,16 +28640,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B59" s="2" t="str">
-        <x:v>GA-R0605</x:v>
+        <x:v>GA-R0618</x:v>
       </x:c>
       <x:c r="C59" s="2" t="str">
-        <x:v>Machine Learning at the Edge: Efficient Utilization of Limited CPU/GPU Resources by Multiplexing</x:v>
+        <x:v>Optimizing GPU Multiplexing for Efficient and Cost-Effective Access to Diverse Large Language Models in GPU Clusters</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E59" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9259361/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10786517/</x:v>
       </x:c>
       <x:c r="F59" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28288,16 +28660,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B60" s="2" t="str">
-        <x:v>GA-R0607</x:v>
+        <x:v>GA-R0620</x:v>
       </x:c>
       <x:c r="C60" s="2" t="str">
-        <x:v>Towards Deterministic End-to-end Latency for Medical AI Systems in NVIDIA Holoscan</x:v>
+        <x:v>Data-Driven Partitioning of Aggregate GPU Power Among GPU (MIG) Partitions</x:v>
       </x:c>
       <x:c r="D60" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E60" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10571631/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11330349/</x:v>
       </x:c>
       <x:c r="F60" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28308,16 +28680,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B61" s="2" t="str">
-        <x:v>GA-R0608</x:v>
+        <x:v>GA-R0621</x:v>
       </x:c>
       <x:c r="C61" s="2" t="str">
-        <x:v>DARIS: An Oversubscribed Spatio-Temporal Scheduler for Real-Time DNN Inference on GPUs</x:v>
+        <x:v>GPU Partitioning &amp; Neural Architecture Sizing for Safety-Driven Sensing in Autonomous Systems</x:v>
       </x:c>
       <x:c r="D61" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E61" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11132423/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10765967/</x:v>
       </x:c>
       <x:c r="F61" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28328,16 +28700,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B62" s="2" t="str">
-        <x:v>GA-R0613</x:v>
+        <x:v>GA-R0622</x:v>
       </x:c>
       <x:c r="C62" s="2" t="str">
-        <x:v>Performance Characterization of LLM Inference under Limited GPU Resources</x:v>
+        <x:v>SGPRS: Seamless GPU Partitioning Real-Time Scheduler for Periodic Deep Learning Workloads</x:v>
       </x:c>
       <x:c r="D62" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E62" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11645315/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10546669/</x:v>
       </x:c>
       <x:c r="F62" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28348,16 +28720,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B63" s="2" t="str">
-        <x:v>GA-R0614</x:v>
+        <x:v>GA-R0624</x:v>
       </x:c>
       <x:c r="C63" s="2" t="str">
-        <x:v>Characterizing GPU Capacity and Computational Cost in Production AI Inference Using a Replica-Centric Measurement Framework</x:v>
+        <x:v>ElasticBatch: A Learning-Augmented Elastic Scheduling System for Batch Inference on MIG</x:v>
       </x:c>
       <x:c r="D63" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E63" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11653193/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10605084/</x:v>
       </x:c>
       <x:c r="F63" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28368,16 +28740,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B64" s="2" t="str">
-        <x:v>GA-R0617</x:v>
+        <x:v>GA-R0628</x:v>
       </x:c>
       <x:c r="C64" s="2" t="str">
-        <x:v>Characterizing Multi-Instance GPU for Machine Learning Workloads</x:v>
+        <x:v>MPTAC: Memory Controller Partitioning and Traffic-Aware Contention Control in GPUs</x:v>
       </x:c>
       <x:c r="D64" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E64" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9835424/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11695654/</x:v>
       </x:c>
       <x:c r="F64" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28388,16 +28760,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B65" s="2" t="str">
-        <x:v>GA-R0618</x:v>
+        <x:v>GA-R0630</x:v>
       </x:c>
       <x:c r="C65" s="2" t="str">
-        <x:v>Optimizing GPU Multiplexing for Efficient and Cost-Effective Access to Diverse Large Language Models in GPU Clusters</x:v>
+        <x:v>FractalGPU: Fair and Elastic GPU Sharing for General-Purpose Computing</x:v>
       </x:c>
       <x:c r="D65" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E65" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10786517/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11619023/</x:v>
       </x:c>
       <x:c r="F65" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28408,16 +28780,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B66" s="2" t="str">
-        <x:v>GA-R0620</x:v>
+        <x:v>GA-R0631</x:v>
       </x:c>
       <x:c r="C66" s="2" t="str">
-        <x:v>Data-Driven Partitioning of Aggregate GPU Power Among GPU (MIG) Partitions</x:v>
+        <x:v>SMOOTH: Scalable Multitask Offloading with Backbone Sharing</x:v>
       </x:c>
       <x:c r="D66" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E66" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11330349/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11578439/</x:v>
       </x:c>
       <x:c r="F66" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28428,16 +28800,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B67" s="2" t="str">
-        <x:v>GA-R0621</x:v>
+        <x:v>GA-R0636</x:v>
       </x:c>
       <x:c r="C67" s="2" t="str">
-        <x:v>GPU Partitioning &amp; Neural Architecture Sizing for Safety-Driven Sensing in Autonomous Systems</x:v>
+        <x:v>Adaptive Kernel Merge and Fusion for Multi-Tenant Inference in Embedded GPUs</x:v>
       </x:c>
       <x:c r="D67" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E67" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10765967/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10384636/</x:v>
       </x:c>
       <x:c r="F67" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28448,16 +28820,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B68" s="2" t="str">
-        <x:v>GA-R0622</x:v>
+        <x:v>GA-R0637</x:v>
       </x:c>
       <x:c r="C68" s="2" t="str">
-        <x:v>SGPRS: Seamless GPU Partitioning Real-Time Scheduler for Periodic Deep Learning Workloads</x:v>
+        <x:v>Leaky DNN: Stealing Deep-Learning Model Secret with GPU Context-Switching Side-Channel</x:v>
       </x:c>
       <x:c r="D68" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E68" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10546669/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9153424/</x:v>
       </x:c>
       <x:c r="F68" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28468,16 +28840,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B69" s="2" t="str">
-        <x:v>GA-R0624</x:v>
+        <x:v>GA-R0638</x:v>
       </x:c>
       <x:c r="C69" s="2" t="str">
-        <x:v>ElasticBatch: A Learning-Augmented Elastic Scheduling System for Batch Inference on MIG</x:v>
+        <x:v>CTXBack: Enabling Low Latency GPU Context Switching via Context Flashback</x:v>
       </x:c>
       <x:c r="D69" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E69" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10605084/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9460478/</x:v>
       </x:c>
       <x:c r="F69" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28488,16 +28860,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B70" s="2" t="str">
-        <x:v>GA-R0628</x:v>
+        <x:v>GA-R0639</x:v>
       </x:c>
       <x:c r="C70" s="2" t="str">
-        <x:v>MPTAC: Memory Controller Partitioning and Traffic-Aware Contention Control in GPUs</x:v>
+        <x:v>Guaranteeing That Multilevel Prioritized DNN Models on an Embedded GPU Have Inference Performance Proportional to Respective Priorities</x:v>
       </x:c>
       <x:c r="D70" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E70" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11695654/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9624962/</x:v>
       </x:c>
       <x:c r="F70" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28508,16 +28880,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B71" s="2" t="str">
-        <x:v>GA-R0630</x:v>
+        <x:v>GA-R0640</x:v>
       </x:c>
       <x:c r="C71" s="2" t="str">
-        <x:v>FractalGPU: Fair and Elastic GPU Sharing for General-Purpose Computing</x:v>
+        <x:v>DyBatch: Efficient Batching and Fair Scheduling for Deep Learning Inference on Time-sharing Devices</x:v>
       </x:c>
       <x:c r="D71" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E71" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11619023/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9139602/</x:v>
       </x:c>
       <x:c r="F71" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28528,16 +28900,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B72" s="2" t="str">
-        <x:v>GA-R0631</x:v>
+        <x:v>GA-R0641</x:v>
       </x:c>
       <x:c r="C72" s="2" t="str">
-        <x:v>SMOOTH: Scalable Multitask Offloading with Backbone Sharing</x:v>
+        <x:v>Efficient Architecture Paradigm for Deep Learning Inference as a Service</x:v>
       </x:c>
       <x:c r="D72" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E72" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11578439/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9391551/</x:v>
       </x:c>
       <x:c r="F72" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28548,16 +28920,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B73" s="2" t="str">
-        <x:v>GA-R0636</x:v>
+        <x:v>GA-R0642</x:v>
       </x:c>
       <x:c r="C73" s="2" t="str">
-        <x:v>Adaptive Kernel Merge and Fusion for Multi-Tenant Inference in Embedded GPUs</x:v>
+        <x:v>HarmonyBatch: Batching multi-SLO DNN Inference with Heterogeneous Serverless Functions</x:v>
       </x:c>
       <x:c r="D73" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E73" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10384636/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10682915/</x:v>
       </x:c>
       <x:c r="F73" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28568,16 +28940,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B74" s="2" t="str">
-        <x:v>GA-R0637</x:v>
+        <x:v>GA-R0644</x:v>
       </x:c>
       <x:c r="C74" s="2" t="str">
-        <x:v>Leaky DNN: Stealing Deep-Learning Model Secret with GPU Context-Switching Side-Channel</x:v>
+        <x:v>Flover: A Temporal Fusion Framework for Efficient Autoregressive Model Parallel Inference</x:v>
       </x:c>
       <x:c r="D74" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E74" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9153424/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10487073/</x:v>
       </x:c>
       <x:c r="F74" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28588,16 +28960,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B75" s="2" t="str">
-        <x:v>GA-R0638</x:v>
+        <x:v>GA-R0646</x:v>
       </x:c>
       <x:c r="C75" s="2" t="str">
-        <x:v>CTXBack: Enabling Low Latency GPU Context Switching via Context Flashback</x:v>
+        <x:v>Adaptive GPU Resource Allocation in Online Scenarios</x:v>
       </x:c>
       <x:c r="D75" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E75" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9460478/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11102455/</x:v>
       </x:c>
       <x:c r="F75" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28608,16 +28980,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B76" s="2" t="str">
-        <x:v>GA-R0639</x:v>
+        <x:v>GA-R0647</x:v>
       </x:c>
       <x:c r="C76" s="2" t="str">
-        <x:v>Guaranteeing That Multilevel Prioritized DNN Models on an Embedded GPU Have Inference Performance Proportional to Respective Priorities</x:v>
+        <x:v>TokenPool-Scheduler: Token-Level GPU Pooling and Resource Slicing for Multi-Model Co-Location</x:v>
       </x:c>
       <x:c r="D76" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E76" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9624962/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11504752/</x:v>
       </x:c>
       <x:c r="F76" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28628,16 +29000,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B77" s="2" t="str">
-        <x:v>GA-R0640</x:v>
+        <x:v>GA-R0648</x:v>
       </x:c>
       <x:c r="C77" s="2" t="str">
-        <x:v>DyBatch: Efficient Batching and Fair Scheduling for Deep Learning Inference on Time-sharing Devices</x:v>
+        <x:v>ServerlessPD: Fast RDMA-Codesigned Disaggregated Prefill-Decoding for Serverless Inference of Large Language Models</x:v>
       </x:c>
       <x:c r="D77" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E77" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9139602/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11169657/</x:v>
       </x:c>
       <x:c r="F77" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28648,16 +29020,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B78" s="2" t="str">
-        <x:v>GA-R0641</x:v>
+        <x:v>GA-R0650</x:v>
       </x:c>
       <x:c r="C78" s="2" t="str">
-        <x:v>Efficient Architecture Paradigm for Deep Learning Inference as a Service</x:v>
+        <x:v>Dissecting Performance Overheads of Confidential Computing on GPU-based Systems</x:v>
       </x:c>
       <x:c r="D78" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E78" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9391551/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11096367/</x:v>
       </x:c>
       <x:c r="F78" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28668,16 +29040,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B79" s="2" t="str">
-        <x:v>GA-R0642</x:v>
+        <x:v>GA-R0654</x:v>
       </x:c>
       <x:c r="C79" s="2" t="str">
-        <x:v>HarmonyBatch: Batching multi-SLO DNN Inference with Heterogeneous Serverless Functions</x:v>
+        <x:v>Workload-Adapted Resource Allocation for LLM Distributed Serving in Serverless Clusters</x:v>
       </x:c>
       <x:c r="D79" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E79" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10682915/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11479931/</x:v>
       </x:c>
       <x:c r="F79" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28688,16 +29060,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B80" s="2" t="str">
-        <x:v>GA-R0644</x:v>
+        <x:v>GA-R0655</x:v>
       </x:c>
       <x:c r="C80" s="2" t="str">
-        <x:v>Flover: A Temporal Fusion Framework for Efficient Autoregressive Model Parallel Inference</x:v>
+        <x:v>Resource Sharing and Security Implications on Machine Learning Inference Accelerators</x:v>
       </x:c>
       <x:c r="D80" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E80" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10487073/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9529641/</x:v>
       </x:c>
       <x:c r="F80" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28708,16 +29080,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B81" s="2" t="str">
-        <x:v>GA-R0646</x:v>
+        <x:v>GA-R0656</x:v>
       </x:c>
       <x:c r="C81" s="2" t="str">
-        <x:v>Adaptive GPU Resource Allocation in Online Scenarios</x:v>
+        <x:v>Breaking the Interaction Wall: A DLPU-Centric Deep Learning Computing System</x:v>
       </x:c>
       <x:c r="D81" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E81" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11102455/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9292952/</x:v>
       </x:c>
       <x:c r="F81" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28728,16 +29100,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B82" s="2" t="str">
-        <x:v>GA-R0647</x:v>
+        <x:v>GA-R0657</x:v>
       </x:c>
       <x:c r="C82" s="2" t="str">
-        <x:v>TokenPool-Scheduler: Token-Level GPU Pooling and Resource Slicing for Multi-Model Co-Location</x:v>
+        <x:v>EdgeServing: Deadline-Aware Multi-DNN Serving at the Edge</x:v>
       </x:c>
       <x:c r="D82" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E82" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11504752/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11662711/</x:v>
       </x:c>
       <x:c r="F82" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28748,16 +29120,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B83" s="2" t="str">
-        <x:v>GA-R0648</x:v>
+        <x:v>GA-R0659</x:v>
       </x:c>
       <x:c r="C83" s="2" t="str">
-        <x:v>ServerlessPD: Fast RDMA-Codesigned Disaggregated Prefill-Decoding for Serverless Inference of Large Language Models</x:v>
+        <x:v>Draco: Dynamic Resource Allocation for Concurrent ML Applications</x:v>
       </x:c>
       <x:c r="D83" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E83" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11169657/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11044818/</x:v>
       </x:c>
       <x:c r="F83" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28768,16 +29140,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B84" s="2" t="str">
-        <x:v>GA-R0650</x:v>
+        <x:v>GA-R0662</x:v>
       </x:c>
       <x:c r="C84" s="2" t="str">
-        <x:v>Dissecting Performance Overheads of Confidential Computing on GPU-based Systems</x:v>
+        <x:v>ArrayPipe: Introducing Job-Array Pipeline Parallelism for High Throughput Model Exploration</x:v>
       </x:c>
       <x:c r="D84" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E84" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11096367/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11044666/</x:v>
       </x:c>
       <x:c r="F84" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28788,16 +29160,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B85" s="2" t="str">
-        <x:v>GA-R0654</x:v>
+        <x:v>GA-R0663</x:v>
       </x:c>
       <x:c r="C85" s="2" t="str">
-        <x:v>Workload-Adapted Resource Allocation for LLM Distributed Serving in Serverless Clusters</x:v>
+        <x:v>Neos: A NVMe-GPUs Direct Vector Service Buffer in User Space</x:v>
       </x:c>
       <x:c r="D85" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E85" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11479931/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10598129/</x:v>
       </x:c>
       <x:c r="F85" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28808,16 +29180,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B86" s="2" t="str">
-        <x:v>GA-R0655</x:v>
+        <x:v>GA-R0666</x:v>
       </x:c>
       <x:c r="C86" s="2" t="str">
-        <x:v>Resource Sharing and Security Implications on Machine Learning Inference Accelerators</x:v>
+        <x:v>Gemini: Enabling Multi-Tenant GPU Sharing Based on Kernel Burst Estimation</x:v>
       </x:c>
       <x:c r="D86" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E86" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9529641/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9566822/</x:v>
       </x:c>
       <x:c r="F86" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28828,16 +29200,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B87" s="2" t="str">
-        <x:v>GA-R0656</x:v>
+        <x:v>GA-R0668</x:v>
       </x:c>
       <x:c r="C87" s="2" t="str">
-        <x:v>Breaking the Interaction Wall: A DLPU-Centric Deep Learning Computing System</x:v>
+        <x:v>Context-Aware Heterogeneous Task Scheduling for Multi-Layered Systems</x:v>
       </x:c>
       <x:c r="D87" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E87" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9292952/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10195463/</x:v>
       </x:c>
       <x:c r="F87" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28848,16 +29220,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B88" s="2" t="str">
-        <x:v>GA-R0657</x:v>
+        <x:v>GA-R0672</x:v>
       </x:c>
       <x:c r="C88" s="2" t="str">
-        <x:v>EdgeServing: Deadline-Aware Multi-DNN Serving at the Edge</x:v>
+        <x:v>Toward Parallel Serving for Vision-Language Models via Modal Decoupling and Scheduling</x:v>
       </x:c>
       <x:c r="D88" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E88" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11662711/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11539390/</x:v>
       </x:c>
       <x:c r="F88" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28868,16 +29240,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B89" s="2" t="str">
-        <x:v>GA-R0659</x:v>
+        <x:v>GA-R0674</x:v>
       </x:c>
       <x:c r="C89" s="2" t="str">
-        <x:v>Draco: Dynamic Resource Allocation for Concurrent ML Applications</x:v>
+        <x:v>CRONUS: Fault-isolated, Secure and High-performance Heterogeneous Computing for Trusted Execution Environment</x:v>
       </x:c>
       <x:c r="D89" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E89" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11044818/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9923810/</x:v>
       </x:c>
       <x:c r="F89" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28888,16 +29260,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B90" s="2" t="str">
-        <x:v>GA-R0662</x:v>
+        <x:v>GA-R0678</x:v>
       </x:c>
       <x:c r="C90" s="2" t="str">
-        <x:v>ArrayPipe: Introducing Job-Array Pipeline Parallelism for High Throughput Model Exploration</x:v>
+        <x:v>SegScope: Probing Fine-grained Interrupts via Architectural Footprints</x:v>
       </x:c>
       <x:c r="D90" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E90" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11044666/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10476480/</x:v>
       </x:c>
       <x:c r="F90" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28908,16 +29280,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B91" s="2" t="str">
-        <x:v>GA-R0663</x:v>
+        <x:v>GA-R0681</x:v>
       </x:c>
       <x:c r="C91" s="2" t="str">
-        <x:v>Neos: A NVMe-GPUs Direct Vector Service Buffer in User Space</x:v>
+        <x:v>Virtualized GPU Offloading for AI Inference: Enabling Deep Learning Frameworks on GPU-less Devices</x:v>
       </x:c>
       <x:c r="D91" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E91" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10598129/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11587741/</x:v>
       </x:c>
       <x:c r="F91" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28928,16 +29300,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B92" s="2" t="str">
-        <x:v>GA-R0666</x:v>
+        <x:v>GA-R0682</x:v>
       </x:c>
       <x:c r="C92" s="2" t="str">
-        <x:v>Gemini: Enabling Multi-Tenant GPU Sharing Based on Kernel Burst Estimation</x:v>
+        <x:v>Edge GPU Virtualization for Cost-Effective Deep Learning Inference in Retail Deployments</x:v>
       </x:c>
       <x:c r="D92" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E92" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9566822/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11715568/</x:v>
       </x:c>
       <x:c r="F92" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28948,16 +29320,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B93" s="2" t="str">
-        <x:v>GA-R0668</x:v>
+        <x:v>GA-R0684</x:v>
       </x:c>
       <x:c r="C93" s="2" t="str">
-        <x:v>Context-Aware Heterogeneous Task Scheduling for Multi-Layered Systems</x:v>
+        <x:v>Dynamic Resource Allocation of Virtualized GPUs and CPUs for Scalable AI Workloads in Containerized Environments</x:v>
       </x:c>
       <x:c r="D93" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E93" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10195463/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/11113647/</x:v>
       </x:c>
       <x:c r="F93" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28968,16 +29340,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B94" s="2" t="str">
-        <x:v>GA-R0672</x:v>
+        <x:v>GA-R0685</x:v>
       </x:c>
       <x:c r="C94" s="2" t="str">
-        <x:v>Toward Parallel Serving for Vision-Language Models via Modal Decoupling and Scheduling</x:v>
+        <x:v>Multi-Tier GPU Virtualization for Deep Learning in Cloud-Edge Systems</x:v>
       </x:c>
       <x:c r="D94" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E94" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11539390/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10122723/</x:v>
       </x:c>
       <x:c r="F94" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -28988,16 +29360,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B95" s="2" t="str">
-        <x:v>GA-R0674</x:v>
+        <x:v>GA-R0686</x:v>
       </x:c>
       <x:c r="C95" s="2" t="str">
-        <x:v>CRONUS: Fault-isolated, Secure and High-performance Heterogeneous Computing for Trusted Execution Environment</x:v>
+        <x:v>Exploiting Interference-aware GPU Container Concurrency Learning from Resource Usage of Application Execution</x:v>
       </x:c>
       <x:c r="D95" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E95" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9923810/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9236964/</x:v>
       </x:c>
       <x:c r="F95" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -29008,16 +29380,16 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B96" s="2" t="str">
-        <x:v>GA-R0678</x:v>
+        <x:v>GA-R0687</x:v>
       </x:c>
       <x:c r="C96" s="2" t="str">
-        <x:v>SegScope: Probing Fine-grained Interrupts via Architectural Footprints</x:v>
+        <x:v>Evaluation of GPU Virtualisation Approaches for Machine Learning Enhanced Debugging of Cloud Orchestration</x:v>
       </x:c>
       <x:c r="D96" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E96" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10476480/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/9465570/</x:v>
       </x:c>
       <x:c r="F96" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
@@ -29028,145 +29400,25 @@
         <x:v>deferred_not_requested</x:v>
       </x:c>
       <x:c r="B97" s="2" t="str">
-        <x:v>GA-R0681</x:v>
+        <x:v>GA-R0688</x:v>
       </x:c>
       <x:c r="C97" s="2" t="str">
-        <x:v>Virtualized GPU Offloading for AI Inference: Enabling Deep Learning Frameworks on GPU-less Devices</x:v>
+        <x:v>SAIndust: A Self-Aware Heterogeneous Computing Framework for Industrial Internet of Things</x:v>
       </x:c>
       <x:c r="D97" s="2" t="str">
         <x:v>IEEE Xplore</x:v>
       </x:c>
       <x:c r="E97" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11587741/</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/10989732/</x:v>
       </x:c>
       <x:c r="F97" s="2" t="str">
-        <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="98" ht="65" customHeight="1">
-      <x:c r="A98" s="2" t="str">
-        <x:v>deferred_not_requested</x:v>
-      </x:c>
-      <x:c r="B98" s="2" t="str">
-        <x:v>GA-R0682</x:v>
-      </x:c>
-      <x:c r="C98" s="2" t="str">
-        <x:v>Edge GPU Virtualization for Cost-Effective Deep Learning Inference in Retail Deployments</x:v>
-      </x:c>
-      <x:c r="D98" s="2" t="str">
-        <x:v>IEEE Xplore</x:v>
-      </x:c>
-      <x:c r="E98" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11715568/</x:v>
-      </x:c>
-      <x:c r="F98" s="2" t="str">
-        <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99" ht="65" customHeight="1">
-      <x:c r="A99" s="2" t="str">
-        <x:v>deferred_not_requested</x:v>
-      </x:c>
-      <x:c r="B99" s="2" t="str">
-        <x:v>GA-R0684</x:v>
-      </x:c>
-      <x:c r="C99" s="2" t="str">
-        <x:v>Dynamic Resource Allocation of Virtualized GPUs and CPUs for Scalable AI Workloads in Containerized Environments</x:v>
-      </x:c>
-      <x:c r="D99" s="2" t="str">
-        <x:v>IEEE Xplore</x:v>
-      </x:c>
-      <x:c r="E99" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/11113647/</x:v>
-      </x:c>
-      <x:c r="F99" s="2" t="str">
-        <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="100" ht="65" customHeight="1">
-      <x:c r="A100" s="2" t="str">
-        <x:v>deferred_not_requested</x:v>
-      </x:c>
-      <x:c r="B100" s="2" t="str">
-        <x:v>GA-R0685</x:v>
-      </x:c>
-      <x:c r="C100" s="2" t="str">
-        <x:v>Multi-Tier GPU Virtualization for Deep Learning in Cloud-Edge Systems</x:v>
-      </x:c>
-      <x:c r="D100" s="2" t="str">
-        <x:v>IEEE Xplore</x:v>
-      </x:c>
-      <x:c r="E100" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10122723/</x:v>
-      </x:c>
-      <x:c r="F100" s="2" t="str">
-        <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="101" ht="65" customHeight="1">
-      <x:c r="A101" s="2" t="str">
-        <x:v>deferred_not_requested</x:v>
-      </x:c>
-      <x:c r="B101" s="2" t="str">
-        <x:v>GA-R0686</x:v>
-      </x:c>
-      <x:c r="C101" s="2" t="str">
-        <x:v>Exploiting Interference-aware GPU Container Concurrency Learning from Resource Usage of Application Execution</x:v>
-      </x:c>
-      <x:c r="D101" s="2" t="str">
-        <x:v>IEEE Xplore</x:v>
-      </x:c>
-      <x:c r="E101" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9236964/</x:v>
-      </x:c>
-      <x:c r="F101" s="2" t="str">
-        <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="102" ht="65" customHeight="1">
-      <x:c r="A102" s="2" t="str">
-        <x:v>deferred_not_requested</x:v>
-      </x:c>
-      <x:c r="B102" s="2" t="str">
-        <x:v>GA-R0687</x:v>
-      </x:c>
-      <x:c r="C102" s="2" t="str">
-        <x:v>Evaluation of GPU Virtualisation Approaches for Machine Learning Enhanced Debugging of Cloud Orchestration</x:v>
-      </x:c>
-      <x:c r="D102" s="2" t="str">
-        <x:v>IEEE Xplore</x:v>
-      </x:c>
-      <x:c r="E102" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/9465570/</x:v>
-      </x:c>
-      <x:c r="F102" s="2" t="str">
-        <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="103" ht="65" customHeight="1">
-      <x:c r="A103" s="2" t="str">
-        <x:v>deferred_not_requested</x:v>
-      </x:c>
-      <x:c r="B103" s="2" t="str">
-        <x:v>GA-R0688</x:v>
-      </x:c>
-      <x:c r="C103" s="2" t="str">
-        <x:v>SAIndust: A Self-Aware Heterogeneous Computing Framework for Industrial Internet of Things</x:v>
-      </x:c>
-      <x:c r="D103" s="2" t="str">
-        <x:v>IEEE Xplore</x:v>
-      </x:c>
-      <x:c r="E103" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/document/10989732/</x:v>
-      </x:c>
-      <x:c r="F103" s="2" t="str">
         <x:v>UNVERIFIED; platform listing is not a subscription guarantee</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra40392cda56c4112"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbe0c826b3c04c6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29422,7 +29674,167 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c54ad398caa462c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcb9ec48088b4ec9"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="65" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="75" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="70" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Record</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>Study</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>Filename</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>Source SHA256</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="70" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>GA-R0006</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>GA-S017</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="str">
+        <x:v>s11390-024-3773-5.md</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="str">
+        <x:v>accepted_new_study</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="str">
+        <x:v>2e387f1599ad6c2fb968c56d604a284491b4e8834df74c7fb2211e79ee62b965</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="70" customHeight="1">
+      <x:c r="A3" s="2" t="str">
+        <x:v>GA-R0037</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>GA-S018</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="str">
+        <x:v>s42514-023-00154-y.md</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="str">
+        <x:v>accepted_new_study</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="str">
+        <x:v>7.0</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="str">
+        <x:v>c1c8557044154d97b0e082a9a7d001883308ad5fef8f0cab98ec52cab62bfe89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="70" customHeight="1">
+      <x:c r="A4" s="2" t="str">
+        <x:v>GA-R0014</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="str">
+        <x:v>GA-S019</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="str">
+        <x:v>s10586-025-05284-2.md</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="str">
+        <x:v>accepted_new_study</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="str">
+        <x:v>7.0</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="str">
+        <x:v>e0eb2886d1c9f029eeb5818ae26c2e50021ba38a736d3d77dfb4302364b03280</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="70" customHeight="1">
+      <x:c r="A5" s="2" t="str">
+        <x:v>GA-X005</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>GA-S020</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="str">
+        <x:v>iGniter_Interference-Aware_GPU_Resource_Provisioning_for_Predictable_DNN_Inference_in_the_Cloud.md</x:v>
+      </x:c>
+      <x:c r="D5" s="2" t="str">
+        <x:v>accepted_new_study</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="str">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="F5" s="2" t="str">
+        <x:v>bdd1f46473d4298c3aa564e42cfda54f65724f7345e57f5b72432115f310e16d</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="70" customHeight="1">
+      <x:c r="A6" s="2" t="str">
+        <x:v>GA-X006</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>GA-S021</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>1-s2.0-S0167739X23003187-main.md</x:v>
+      </x:c>
+      <x:c r="D6" s="2" t="str">
+        <x:v>accepted_new_study</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="str">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F6" s="2" t="str">
+        <x:v>7e82b1df848b5d798f68cf11602de9e4b715b3d0aabe5e0ea99183230695e55e</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="70" customHeight="1">
+      <x:c r="A7" s="2" t="str">
+        <x:v>GA-X007</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>GA-S001</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>3768622.md</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="str">
+        <x:v>preferred_journal_version_same_study</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="str">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="F7" s="2" t="str">
+        <x:v>6dfba38d0d9567367f29c9773cec77db37499e47d83ac5bb6119aa89d8726389</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5806c7b7af304478"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>